<commit_message>
chore: backlog 43/44/42/45/30 — cleanup developer_notes, zasady, task type
</commit_message>
<xml_diff>
--- a/solutions/bi/TwrKarty/TwrKarty_plan.xlsx
+++ b/solutions/bi/TwrKarty/TwrKarty_plan.xlsx
@@ -700,6 +700,11 @@
           <t>Typ kartoteki towarowej</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Enumeracja: wartosc 6 nieznana. Blokuje draft — zidentyfikuj znaczenie przed SQL (docs_search lub CDN.Obiekty).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1145,6 +1150,11 @@
           <t>4 wartosci — znaczenie wymaga dokumentacji</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Enumeracja bez CASE: wartosci 0,2,3,4. Zidentyfikuj znaczenie lub zastosuj CASE z ELSE 'Nieznane('+CAST AS VARCHAR+')'.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1785,6 +1795,11 @@
           <t>3 wartosci — cena 1/3/6</t>
         </is>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Typ/enumeracja (1,3,6) — 'bez zmian' niewystarczajace w BI. Wymagany CASE z etykietami.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1825,6 +1840,11 @@
           <t>FK do tabeli JM — 6 wartosci</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>FK do JM, 6 wartosci. Czy istnieje tabela JM do dekodowania? Jesli tak — dodaj JOIN zamiast surowego ID.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1865,6 +1885,11 @@
           <t>Typ domyslnego dostawcy</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Wartosci 0–4 — nie jest flaga 0/1. Wymagany CASE z etykietami (typ domyslnego dostawcy).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3165,6 +3190,11 @@
           <t>Kod katalogu — 4 wartosci w tym puste</t>
         </is>
       </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Znaczenie niewyjasnione (P-100, EAN-podobne, puste). Wyjasniej semantyke przed draftem.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3510,6 +3540,11 @@
           <t>Timestamp ostatniej modyfikacji (liczba)</t>
         </is>
       </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Suffiks L/O/C — roznica semantyczna? Trzy timestampy modyfikacji wymagaja wyjasnienia znaczenia.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3545,6 +3580,11 @@
           <t>Timestamp modyfikacji O</t>
         </is>
       </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>jw. — patrz Twr_LastModL.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3580,6 +3620,11 @@
           <t>Timestamp modyfikacji C</t>
         </is>
       </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>jw. — patrz Twr_LastModL.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3940,6 +3985,11 @@
           <t>Typ kosztu: 2 wartosci</t>
         </is>
       </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Flaga 0/1 — powinna miec CASE jak inne flagi w planie. Zmien transformacje na CASE 1=Tak 0=Nie.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4420,6 +4470,11 @@
           <t>FK do CDN.CechyKlasy (typ 192) — 2 wartosci</t>
         </is>
       </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>FK do CechyKlasy, 2 wartosci (0 i 1). Co reprezentuje wartosc 1? Weryfikuj przez docs_search lub CDN.Obiekty typ 192.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -5320,6 +5375,11 @@
           <t>UWAGA: Twr_Aktywna stala=0 — status aktywnosci tu</t>
         </is>
       </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>CASE 1=Tak 0=Nie — proponuje 1='Archiwalny' 0='Aktywny' (semantycznie spojne z nazwa pola i anomalia Twr_Aktywna).</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -6825,6 +6885,11 @@
           <t>Flaga dostepnosci PIA</t>
         </is>
       </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Wartosci 0 i 8 — NIE jest flaga 0/1. Znaczenie 8 nieznane. Wymagany CASE przed draftem.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -7230,6 +7295,11 @@
           <t>FK do systemu MRP — 1172 roznych wartosci</t>
         </is>
       </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>FK, 1172 distinct wartosci. Czy istnieje tabela CDN dla MRP? Jesli tak — JOIN zamiast surowego ID. Jesli nie — zachowaj z adnotacja.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -7465,6 +7535,11 @@
           <t>3 wartosci — typ zezwolenia</t>
         </is>
       </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Enumeracja 3-wartosciowa (0,1,2) — wymaga CASE z etykietami. 'bez zmian' nie wystarczy.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -8130,6 +8205,11 @@
           <t>Kategoria domowa towaru z hierarchii grup</t>
         </is>
       </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>JOIN z TGD_GIDTyp=-16 (wartosc ujemna). Zweryfikuj czy typ -16 istnieje w CDN.Obiekty. Niestandardowe.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -8233,6 +8313,11 @@
       <c r="H200" t="inlineStr">
         <is>
           <t>Producent towaru jako kontrahent</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>JOIN tylko na Knt_GIDNumer — brakuje warunku Knt_GIDTyp = Twr_PrdTyp (=32). Dwuczescowy klucz wymagany (konwencja JOIN KntKarty).</t>
         </is>
       </c>
     </row>

</xml_diff>